<commit_message>
📊 Daily DSE update
</commit_message>
<xml_diff>
--- a/dse_market_summary.xlsx
+++ b/dse_market_summary.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I579"/>
+  <dimension ref="A1:I580"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27657,6 +27657,53 @@
         </is>
       </c>
     </row>
+    <row r="580">
+      <c r="A580" s="3" t="inlineStr">
+        <is>
+          <t>236,459,490</t>
+        </is>
+      </c>
+      <c r="B580" s="3" t="inlineStr">
+        <is>
+          <t>2,072.01385</t>
+        </is>
+      </c>
+      <c r="C580" s="3" t="inlineStr">
+        <is>
+          <t>Sep 13, 2026</t>
+        </is>
+      </c>
+      <c r="D580" s="3" t="inlineStr">
+        <is>
+          <t>5,418.55361</t>
+        </is>
+      </c>
+      <c r="E580" s="3" t="inlineStr">
+        <is>
+          <t>-23.29665</t>
+        </is>
+      </c>
+      <c r="F580" s="3" t="inlineStr">
+        <is>
+          <t>-96.61455</t>
+        </is>
+      </c>
+      <c r="G580" s="3" t="inlineStr">
+        <is>
+          <t>5,713.183</t>
+        </is>
+      </c>
+      <c r="H580" s="3" t="inlineStr">
+        <is>
+          <t>6,862,972.350</t>
+        </is>
+      </c>
+      <c r="I580" s="3" t="inlineStr">
+        <is>
+          <t>182,186</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>